<commit_message>
Restyle class work files in black, white and blue
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ViSVrkfNYmVSDoY4z54Vze
</commit_message>
<xml_diff>
--- a/research-register/ChatGPT_Claude_Courses_Register_Excel2013.xlsx
+++ b/research-register/ChatGPT_Claude_Courses_Register_Excel2013.xlsx
@@ -18,11 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
-    <numFmt numFmtId="165" formatCode="+#,##0;[Red]-#,##0;0"/>
+    <numFmt numFmtId="165" formatCode="[Blue]+#,##0;[Black]-#,##0;0"/>
+    <numFmt numFmtId="166" formatCode="+#,##0;-#,##0;0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,7 +34,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F4E78"/>
+      <color rgb="001A56DB"/>
       <sz val="16"/>
     </font>
     <font>
@@ -41,19 +42,16 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
-      <color rgb="000563C1"/>
+      <color rgb="001A56DB"/>
       <u val="single"/>
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E78"/>
+      <color rgb="001A56DB"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00404040"/>
+      <color rgb="00000000"/>
     </font>
   </fonts>
   <fills count="5">
@@ -64,18 +62,16 @@
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
+      <patternFill patternType="solid"/>
+    </fill>
+    <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="00EEF4FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
+        <fgColor rgb="001A56DB"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,16 +85,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00A6A6A6"/>
+        <color rgb="00000000"/>
       </left>
       <right style="thin">
-        <color rgb="00A6A6A6"/>
+        <color rgb="00000000"/>
       </right>
       <top style="thin">
-        <color rgb="00A6A6A6"/>
+        <color rgb="00000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00A6A6A6"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
   </borders>
@@ -149,23 +145,23 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -927,7 +923,7 @@
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>Variance = Actual results of registrants − Projected target (red / minus = below target)</t>
+          <t>Variance = Actual results of registrants − Projected target (minus = below target)</t>
         </is>
       </c>
     </row>

</xml_diff>